<commit_message>
Add complete SKEMA professors profile audit & Front Office LOR strategy + fix CTM Excel model inputs
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cours/S1_CTM/CTM_Exercise_1_Model.xlsx
+++ b/cours/S1_CTM/CTM_Exercise_1_Model.xlsx
@@ -566,7 +566,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>1. INPUT FINANCIAL DATA (EUR m)</t>
+          <t>1. INPUT FINANCIAL DATA (EUR m) — Exact figures from Exercise 1.docx</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
@@ -589,10 +589,10 @@
         <v>500</v>
       </c>
       <c r="D5" s="7" t="n">
+        <v>365</v>
+      </c>
+      <c r="E5" s="7" t="n">
         <v>300</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>400</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>400</v>
@@ -610,16 +610,16 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>820</v>
+        <v>750</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>400</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>120</v>
@@ -670,10 +670,10 @@
         <v>100</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>49.3</v>
+        <v>60</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>10</v>
@@ -691,16 +691,16 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>71.09999999999999</v>
+        <v>65</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>180</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>34.5</v>
+        <v>36</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>80</v>
@@ -718,16 +718,16 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>120.3</v>
+        <v>110</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>90</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>40.3</v>
+        <v>42</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>25</v>
@@ -745,19 +745,19 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="C11" s="7" t="n">
         <v>40</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>60</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>20</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -772,19 +772,19 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -799,19 +799,19 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>4</v>
-      </c>
       <c r="F13" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>

</xml_diff>